<commit_message>
new infra of multiset ansatz
</commit_message>
<xml_diff>
--- a/test/test_Holstein_5/plot/Holstein5_16bd_singleset.xlsx
+++ b/test/test_Holstein_5/plot/Holstein5_16bd_singleset.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6F0E4D5-E37B-4016-AB62-2A4B29083FFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7480F73-7A90-443E-82E3-6614052E22E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2040" yWindow="3440" windowWidth="19200" windowHeight="10140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>